<commit_message>
OZON пенки: добавлена FARMSTAY Collagen Pure Cleansing Foam 180ml (остаток 515)
Способ применения — с офиц. сайта FARMSTAY (RU), состав английский (INCI из
выгрузки ВБ), производитель Myungin Cosmetics, прочие поля по общим правилам.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_cleanser_cards/ozon_cleansers_2026-08-06.xlsx
+++ b/outputs/ozon_cleanser_cards/ozon_cleansers_2026-08-06.xlsx
@@ -1922,55 +1922,183 @@
       <c r="AY7" s="4" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>FARMSTAY - Collagen Pure Cleansing Foam [180ml]</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Корейская пенка для умывания лица увлажняющая FARMSTAY, 180 мл</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
+      <c r="F8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
       <c r="I8" s="6" t="n"/>
-      <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
-      <c r="L8" s="4" t="n"/>
-      <c r="M8" s="4" t="n"/>
-      <c r="N8" s="4" t="n"/>
-      <c r="O8" s="4" t="n"/>
-      <c r="P8" s="4" t="n"/>
-      <c r="Q8" s="4" t="n"/>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>2039455156657</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>3304990000 - Прочие косметические средства или средства для макияжа и средства для ухода за кожей (кроме лекарственных), включая средства против загара или для загара; средства для маникюра или педикюра</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>224</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>190</v>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/1.webp</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/2.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/3.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/4.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/5.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/6.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/7.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/8.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/9.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/10.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/11.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/12.webp;https://basket-14.wbbasket.ru/vol2074/part207476/207476777/images/big/13.webp</t>
+        </is>
+      </c>
       <c r="R8" s="4" t="n"/>
-      <c r="S8" s="4" t="n"/>
-      <c r="T8" s="4" t="n"/>
-      <c r="U8" s="4" t="n"/>
-      <c r="V8" s="4" t="n"/>
-      <c r="W8" s="4" t="n"/>
-      <c r="X8" s="4" t="n"/>
-      <c r="Y8" s="4" t="n"/>
-      <c r="Z8" s="4" t="n"/>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>Средство для умывания</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>farmstay</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>FARMSTAY - Collagen Pure Cleansing Foam [180ml]</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="X8" s="4" t="inlineStr">
+        <is>
+          <t>Water;Stearic Acid;Lauric Acid;Potasium Hydroxide;Glycine;Myristic Acid;Cocamidopropyl Bataine;Polysorbate 60;Glycol Distearate;Glyceryl Stearate;PEG-100 Glyceryl Stearate;Methyl Paraben;Propyl Paraben;Collagen Filtrate (180mg);Olive Extract;Green Tea Extract;Perfume</t>
+        </is>
+      </c>
+      <c r="Y8" s="4" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <v>1095</v>
+      </c>
       <c r="AA8" s="4" t="n"/>
       <c r="AB8" s="4" t="n"/>
-      <c r="AC8" s="4" t="n"/>
+      <c r="AC8" s="4" t="inlineStr">
+        <is>
+          <t>Myungin Cosmetics Co., Ltd.</t>
+        </is>
+      </c>
       <c r="AD8" s="4" t="n"/>
       <c r="AE8" s="4" t="n"/>
-      <c r="AF8" s="4" t="n"/>
+      <c r="AF8" s="4" t="inlineStr">
+        <is>
+          <t>Регулярное очищение лица – это базовый уход за лицом и первый этап корейской системы, позволяющей поддержать здоровье и естественную красоту кожи. Пенка для умывания лица от бренда FARMSTAY отлично подойдет для этой задачи, ведь она мягко убирает все естественные и внешние загрязнения, смывает макияж, растворяет выделившийся за день себум. Это эффективное, но деликатное средство для умывания со специальной омолаживающей формулой. 
+Farmstay Корейская умывалка для лица коллаген не содержит агрессивных очищающих компонентов, которые могли бы навредить коже или вызвать сухость. Наоборот, коллагеновая пенка для умывания дает базовое увлажнение, восстанавливает обмен веществ эпидермиса и хорошо помогает от прыщей, очищая поры от накопившегося себума. 
+Пена для умывания FARMSTAY Collagen Pure Cleansing Foam подходит для ежедневного использования и любого типа кожи, включая чувствительную и проблемную кожу. Включите это средство для умывания в утренний и вечерний уход за лицом, а также используйте для снятия макияжа (можно наносить в два этапа, чтобы смыть стойкую косметику).
+Одно из главных активных веществ в составе продукта – это коллаген для лица. Пенка для умывания восполняет недостаток коллагена в коже, возвращая ей эластичность и упругость. Если коллаген не вырабатывается организмом в нужном количестве, то на лице становятся заметны возрастные изменения: пенка для умывания Корея с коллагеном позволяет поддержать естественную красоту и молодость кожи. Качественное очищение лица, которое не пересушивает кожу, помогает достичь максимального результата в создании ровной кожи без прыщей, пигментации и морщин!
+В отличие от обычных гелей и очищающих продуктов, FARMSTAY Collagen Pure Cleansing Foam увлажняет кожу, спасает ее от обезвоженности и работает как пенка для умывания от прыщей. В ней нет агрессивных кислот, противопоказанных сухой и чувствительной коже, но при этом пенка для лица хорошо очищает поры, а экстракт зеленого чая помогает справиться с воспалениями.</t>
+        </is>
+      </c>
       <c r="AG8" s="4" t="n"/>
       <c r="AH8" s="4" t="n"/>
       <c r="AI8" s="4" t="n"/>
-      <c r="AJ8" s="4" t="n"/>
-      <c r="AK8" s="4" t="n"/>
-      <c r="AL8" s="4" t="n"/>
-      <c r="AM8" s="4" t="n"/>
+      <c r="AJ8" s="4" t="inlineStr">
+        <is>
+          <t>Возьмите умеренное количество пенки на ладонь и вспеньте с небольшим количеством воды до плотной пены. Мягко распределите по всему лицу лёгкими массирующими движениями, избегая области вокруг глаз. Тщательно смойте тёплой водой и продолжите привычный уход. Подходит для ежедневного применения.</t>
+        </is>
+      </c>
+      <c r="AK8" s="4" t="inlineStr">
+        <is>
+          <t>Коллаген;Растительный экстракт</t>
+        </is>
+      </c>
+      <c r="AL8" s="4" t="inlineStr">
+        <is>
+          <t>пенка</t>
+        </is>
+      </c>
+      <c r="AM8" s="4" t="inlineStr">
+        <is>
+          <t>Для всех типов кожи;Для сухой кожи;Для нормальной кожи</t>
+        </is>
+      </c>
       <c r="AN8" s="4" t="n"/>
-      <c r="AO8" s="4" t="n"/>
-      <c r="AP8" s="4" t="n"/>
-      <c r="AQ8" s="4" t="n"/>
-      <c r="AR8" s="4" t="n"/>
-      <c r="AS8" s="4" t="n"/>
-      <c r="AT8" s="4" t="n"/>
-      <c r="AU8" s="4" t="n"/>
+      <c r="AO8" s="4" t="inlineStr">
+        <is>
+          <t>Очищение;Увлажнение;Питание</t>
+        </is>
+      </c>
+      <c r="AP8" s="4" t="inlineStr">
+        <is>
+          <t>Лицо</t>
+        </is>
+      </c>
+      <c r="AQ8" s="4" t="inlineStr">
+        <is>
+          <t>Подходит для ежедневного применения</t>
+        </is>
+      </c>
+      <c r="AR8" s="4" t="inlineStr">
+        <is>
+          <t>Взрослая</t>
+        </is>
+      </c>
+      <c r="AS8" s="4" t="inlineStr">
+        <is>
+          <t>Для любого возраста</t>
+        </is>
+      </c>
+      <c r="AT8" s="4" t="inlineStr">
+        <is>
+          <t>Южная Корея</t>
+        </is>
+      </c>
+      <c r="AU8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="AV8" s="4" t="n"/>
-      <c r="AW8" s="4" t="n"/>
+      <c r="AW8" s="4" t="inlineStr">
+        <is>
+          <t>Не опасен</t>
+        </is>
+      </c>
       <c r="AX8" s="4" t="n"/>
       <c r="AY8" s="4" t="n"/>
     </row>

</xml_diff>